<commit_message>
feat: log-work modal improvements and HQ reports
- Checklist state persistence: save/restore checked items via Firestore
- Fix arrival time race condition: skip async restore if user already edited fields
- Fix maintenance recommendation: save date-only entries, restore date as string for input display
- Fix sign-off button: use z.coerce.date() for maintenance date validation
- HQ reports: machine reliability, parts consumption, resolution times, store comparison, technician performance, ticket analysis
- New lib/actions/hq-reports.ts server actions
- New lib/client-cache.ts utility
</commit_message>
<xml_diff>
--- a/test-data/machines-test.xlsx
+++ b/test-data/machines-test.xlsx
@@ -397,11 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E57"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="34.83203125" customWidth="1"/>
     <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="36.83203125" customWidth="1"/>
   </cols>
@@ -425,10 +425,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>CRS-2021-0001</v>
+        <v>IPL-2022-0001</v>
       </c>
       <c r="B2" t="str">
-        <v>Crescendo</v>
+        <v>iPilot Machine</v>
       </c>
       <c r="C2" t="str">
         <v>Blue Waters Hotels &amp; Resorts</v>
@@ -442,16 +442,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ESP-2019-0042</v>
+        <v>EGR-2021-0002</v>
       </c>
       <c r="B3" t="str">
-        <v>Espresso</v>
+        <v>EGRO Machine</v>
       </c>
       <c r="C3" t="str">
-        <v>Carib Coffee Co</v>
+        <v>Blue Waters Hotels &amp; Resorts</v>
       </c>
       <c r="D3" t="str">
-        <v>Counter 1</v>
+        <v>Restaurant Bar</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -459,33 +459,33 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>GRD-2020-0015</v>
+        <v>WTR-2023-0003</v>
       </c>
       <c r="B4" t="str">
-        <v>Grinder</v>
+        <v>Water Machine</v>
       </c>
       <c r="C4" t="str">
-        <v>Carib Coffee Co</v>
+        <v>Blue Waters Hotels &amp; Resorts</v>
       </c>
       <c r="D4" t="str">
-        <v>Counter 1</v>
+        <v>Back Kitchen</v>
       </c>
       <c r="E4" t="str">
-        <v>Burr replaced Mar 2025</v>
+        <v>Filter replaced Jan 2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CRS-2022-0018</v>
+        <v>CRS-2020-0004</v>
       </c>
       <c r="B5" t="str">
-        <v>Crescendo</v>
+        <v>Crescendo Machine</v>
       </c>
       <c r="C5" t="str">
-        <v>Trini Roast Ltd</v>
+        <v>Carib Coffee Co</v>
       </c>
       <c r="D5" t="str">
-        <v>Front Counter</v>
+        <v>Counter 1</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -493,101 +493,101 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ESP-2021-0033</v>
+        <v>RAN-2019-0005</v>
       </c>
       <c r="B6" t="str">
-        <v>Espresso</v>
+        <v>Rancilio Espresso Machine</v>
       </c>
       <c r="C6" t="str">
-        <v>Island Brew Café</v>
+        <v>Carib Coffee Co</v>
       </c>
       <c r="D6" t="str">
-        <v>Bar Area</v>
+        <v>Counter 2</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>Pump seal replaced Sep 2025</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>GRD-2021-0009</v>
+        <v>BGD-2021-0006</v>
       </c>
       <c r="B7" t="str">
-        <v>Grinder</v>
+        <v>BUNN Grinder</v>
       </c>
       <c r="C7" t="str">
-        <v>Island Brew Café</v>
+        <v>Carib Coffee Co</v>
       </c>
       <c r="D7" t="str">
-        <v>Bar Area</v>
+        <v>Counter 1</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>Burr replaced Mar 2025</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>CRS-2020-0027</v>
+        <v>IPL-2022-0007</v>
       </c>
       <c r="B8" t="str">
-        <v>Crescendo</v>
+        <v>iPilot Machine</v>
       </c>
       <c r="C8" t="str">
-        <v>Coffee Republic</v>
+        <v>Trini Roast Ltd</v>
       </c>
       <c r="D8" t="str">
-        <v>Main Floor</v>
+        <v>Front Counter</v>
       </c>
       <c r="E8" t="str">
-        <v>Older unit, monitor closely</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ESP-2023-0005</v>
+        <v>CRS-2022-0008</v>
       </c>
       <c r="B9" t="str">
-        <v>Espresso</v>
+        <v>Crescendo Machine</v>
       </c>
       <c r="C9" t="str">
-        <v>Savana Grande Hotel</v>
+        <v>Trini Roast Ltd</v>
       </c>
       <c r="D9" t="str">
-        <v>Restaurant</v>
+        <v>Back Counter</v>
       </c>
       <c r="E9" t="str">
-        <v>New install Jan 2023</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>CRS-2018-0044</v>
+        <v>SMW-2023-0009</v>
       </c>
       <c r="B10" t="str">
-        <v>Crescendo</v>
+        <v>Smartwave Brewer Machine</v>
       </c>
       <c r="C10" t="str">
-        <v>Tobago Plantation Café</v>
+        <v>Trini Roast Ltd</v>
       </c>
       <c r="D10" t="str">
-        <v>Counter</v>
+        <v>Staff Break Room</v>
       </c>
       <c r="E10" t="str">
-        <v>Due for descale</v>
+        <v>New install Mar 2023</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ESP-2022-0011</v>
+        <v>RAN-2021-0010</v>
       </c>
       <c r="B11" t="str">
-        <v>Espresso</v>
+        <v>Rancilio Espresso Machine</v>
       </c>
       <c r="C11" t="str">
-        <v>Maracas Bay Resort</v>
+        <v>Island Brew Café</v>
       </c>
       <c r="D11" t="str">
-        <v>Pool Bar</v>
+        <v>Bar Area</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -595,16 +595,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>GRD-2022-0003</v>
+        <v>BKY-2022-0011</v>
       </c>
       <c r="B12" t="str">
-        <v>Grinder</v>
+        <v>BUNN Kyro Grinder</v>
       </c>
       <c r="C12" t="str">
-        <v>Maracas Bay Resort</v>
+        <v>Island Brew Café</v>
       </c>
       <c r="D12" t="str">
-        <v>Pool Bar</v>
+        <v>Bar Area</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -612,16 +612,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CRS-2021-0059</v>
+        <v>WTR-2021-0012</v>
       </c>
       <c r="B13" t="str">
-        <v>Crescendo</v>
+        <v>Water Machine</v>
       </c>
       <c r="C13" t="str">
-        <v>Pan Espresso Bar</v>
+        <v>Island Brew Café</v>
       </c>
       <c r="D13" t="str">
-        <v>Station 1</v>
+        <v>Kitchen</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -629,33 +629,33 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ESP-2021-0060</v>
+        <v>CRS-2020-0013</v>
       </c>
       <c r="B14" t="str">
-        <v>Espresso</v>
+        <v>Crescendo Machine</v>
       </c>
       <c r="C14" t="str">
-        <v>Pan Espresso Bar</v>
+        <v>Coffee Republic</v>
       </c>
       <c r="D14" t="str">
-        <v>Station 2</v>
+        <v>Main Floor</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>Older unit — monitor closely</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CRS-2019-0031</v>
+        <v>SIL-2021-0014</v>
       </c>
       <c r="B15" t="str">
-        <v>Crescendo</v>
+        <v>Silvia Espresso Machine</v>
       </c>
       <c r="C15" t="str">
-        <v>Gulf City Mall Food Court</v>
+        <v>Coffee Republic</v>
       </c>
       <c r="D15" t="str">
-        <v>Unit A</v>
+        <v>Brew Station</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -663,16 +663,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ESP-2020-0022</v>
+        <v>BGD-2022-0015</v>
       </c>
       <c r="B16" t="str">
-        <v>Espresso</v>
+        <v>BUNN Grinder</v>
       </c>
       <c r="C16" t="str">
-        <v>Hyatt Regency Trinidad</v>
+        <v>Coffee Republic</v>
       </c>
       <c r="D16" t="str">
-        <v>Restaurant</v>
+        <v>Brew Station</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -680,92 +680,704 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>GRD-2020-0016</v>
+        <v>EGR-2023-0016</v>
       </c>
       <c r="B17" t="str">
-        <v>Grinder</v>
+        <v>EGRO Machine</v>
       </c>
       <c r="C17" t="str">
-        <v>Hyatt Regency Trinidad</v>
+        <v>Savana Grande Hotel</v>
       </c>
       <c r="D17" t="str">
         <v>Restaurant</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>New install Jan 2023</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>CRS-2023-0008</v>
+        <v>IPL-2021-0017</v>
       </c>
       <c r="B18" t="str">
-        <v>Crescendo</v>
+        <v>iPilot Machine</v>
       </c>
       <c r="C18" t="str">
-        <v>Meridian Coffee House</v>
+        <v>Savana Grande Hotel</v>
       </c>
       <c r="D18" t="str">
-        <v>Main Bar</v>
+        <v>Lobby Café</v>
       </c>
       <c r="E18" t="str">
-        <v>New install</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>OTH-2021-0037</v>
+        <v>BSV-2022-0018</v>
       </c>
       <c r="B19" t="str">
-        <v>Other</v>
+        <v>BUNN Server</v>
       </c>
       <c r="C19" t="str">
-        <v>Cocoa Lounge Bar</v>
+        <v>Savana Grande Hotel</v>
       </c>
       <c r="D19" t="str">
-        <v>VIP Area</v>
+        <v>Conference Room</v>
       </c>
       <c r="E19" t="str">
-        <v>Cold brew tower</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>CRS-2022-0013</v>
+        <v>CRS-2018-0019</v>
       </c>
       <c r="B20" t="str">
-        <v>Crescendo</v>
+        <v>Crescendo Machine</v>
       </c>
       <c r="C20" t="str">
-        <v>Port of Spain Marriott</v>
+        <v>Tobago Plantation Café</v>
       </c>
       <c r="D20" t="str">
-        <v>Lobby Café</v>
+        <v>Counter</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>Due for descale</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>ESP-2023-0002</v>
+        <v>RAN-2020-0020</v>
       </c>
       <c r="B21" t="str">
-        <v>Espresso</v>
+        <v>Rancilio Espresso Machine</v>
       </c>
       <c r="C21" t="str">
+        <v>Tobago Plantation Café</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Counter</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>SIL-2022-0021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Silvia Espresso Machine</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Maracas Bay Resort</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Pool Bar</v>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>BGD-2022-0022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>BUNN Grinder</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Maracas Bay Resort</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Pool Bar</v>
+      </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>WTR-2020-0023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Water Machine</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Maracas Bay Resort</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Kitchen</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Scale build-up noted</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>RAN-2021-0024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Rancilio Espresso Machine</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Pan Espresso Bar</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Station 1</v>
+      </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>BKY-2021-0025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>BUNN Kyro Grinder</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Pan Espresso Bar</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Station 1</v>
+      </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>IPL-2022-0026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>iPilot Machine</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Pan Espresso Bar</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Station 2</v>
+      </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>CRS-2021-0027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Crescendo Machine</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Chaguanas Trade Centre</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Food Court</v>
+      </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>BRW-2022-0028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Brewer Machine</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Chaguanas Trade Centre</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Food Court</v>
+      </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>CRS-2019-0029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Crescendo Machine</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Gulf City Mall Food Court</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Unit A</v>
+      </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>SAM-2021-0030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Samremo Grinder</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Gulf City Mall Food Court</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Unit A</v>
+      </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>WTR-2022-0031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Water Machine</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Gulf City Mall Food Court</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Unit B</v>
+      </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>EGR-2020-0032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>EGRO Machine</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Hyatt Regency Trinidad</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Restaurant</v>
+      </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>BGD-2020-0033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>BUNN Grinder</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Hyatt Regency Trinidad</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Restaurant</v>
+      </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>IPL-2021-0034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>iPilot Machine</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Hyatt Regency Trinidad</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Lobby Lounge</v>
+      </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>BRW-2022-0035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Brewer Machine</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Hyatt Regency Trinidad</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Conference Suite</v>
+      </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>CRS-2022-0036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Crescendo Machine</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Starlite Hotel</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Breakfast Area</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>RAN-2021-0037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Rancilio Espresso Machine</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Starlite Hotel</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Breakfast Area</v>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>IPL-2023-0038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>iPilot Machine</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Meridian Coffee House</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Main Bar</v>
+      </c>
+      <c r="E39" t="str">
+        <v>New install</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>SIL-2022-0039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Silvia Espresso Machine</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Meridian Coffee House</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Main Bar</v>
+      </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>BKY-2022-0040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>BUNN Kyro Grinder</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Meridian Coffee House</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Main Bar</v>
+      </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>NIT-2021-0041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Nitron RMV</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Cocoa Lounge Bar</v>
+      </c>
+      <c r="D42" t="str">
+        <v>VIP Area</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Cold brew system</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>WTR-2021-0042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Water Machine</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Cocoa Lounge Bar</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Back Bar</v>
+      </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>EGR-2022-0043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>EGRO Machine</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Port of Spain Marriott</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Lobby Café</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>IPL-2022-0044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>iPilot Machine</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Port of Spain Marriott</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Executive Lounge</v>
+      </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>BSV-2021-0045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>BUNN Server</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Port of Spain Marriott</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Meeting Rooms</v>
+      </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>CRS-2021-0046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Crescendo Machine</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Arima Roasters</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Shop Floor</v>
+      </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>BRW-2020-0047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Brewer Machine</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Arima Roasters</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Shop Floor</v>
+      </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>SAM-2022-0048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Samremo Grinder</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Arima Roasters</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Shop Floor</v>
+      </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>RAN-2022-0049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Rancilio Espresso Machine</v>
+      </c>
+      <c r="C50" t="str">
+        <v>River Estate Café</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Counter</v>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>BGD-2021-0050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>BUNN Grinder</v>
+      </c>
+      <c r="C51" t="str">
+        <v>River Estate Café</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Counter</v>
+      </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>IPL-2023-0051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>iPilot Machine</v>
+      </c>
+      <c r="C52" t="str">
         <v>Airport Lounge TT</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D52" t="str">
         <v>Terminal 2</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>EGR-2022-0052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>EGRO Machine</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Airport Lounge TT</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Terminal 1</v>
+      </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>CRS-2021-0053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Crescendo Machine</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Airport Lounge TT</v>
+      </c>
+      <c r="D54" t="str">
+        <v>VIP Lounge</v>
+      </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>SMW-2022-0054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Smartwave Brewer Machine</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Couva Central Mall</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Food Court A</v>
+      </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>BGD-2023-0055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>BUNN Grinder</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Couva Central Mall</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Food Court A</v>
+      </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>WTR-2022-0056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Water Machine</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Couva Central Mall</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Food Court B</v>
+      </c>
+      <c r="E57" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>